<commit_message>
Update TS3_mapping.xlsx via Streamlit
</commit_message>
<xml_diff>
--- a/TS3_mapping.xlsx
+++ b/TS3_mapping.xlsx
@@ -1565,9 +1565,10 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Spectrum-6 in Flash Recovery Mode. 
+          <t xml:space="preserve">Spectrum-6 in Flash Recovery Mode. 
 Suspect ASIC issue.
-Tried master PDB then pass. Replacing with new PDB to retest.</t>
+Tried master PDB then pass. Replacing with new PDB to retest.
+29-SEP: Passed with new PDB - &gt; retets on PDB station </t>
         </is>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -2729,8 +2730,9 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Spectrum-6 in Flash Recovery Mode. 
-Suspect ASIC issue.</t>
+          <t xml:space="preserve">Spectrum-6 in Flash Recovery Mode. 
+Suspect ASIC issue.
+NV : share details </t>
         </is>
       </c>
       <c r="Q41" t="inlineStr"/>

</xml_diff>